<commit_message>
updated liver gene to correct spelling
</commit_message>
<xml_diff>
--- a/Data/Excel/pcr-data-mix.xlsx
+++ b/Data/Excel/pcr-data-mix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cornellprod-my.sharepoint.com/personal/cjm423_cornell_edu/Documents/study-1-march25/MIX/Data/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="930" documentId="8_{B7E12F50-AE19-4325-ACC3-C71BB40EE95D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D30DCBB-1237-47DA-B187-317DCA48C6B0}"/>
+  <xr:revisionPtr revIDLastSave="1017" documentId="8_{B7E12F50-AE19-4325-ACC3-C71BB40EE95D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65E4AD4F-C410-46EC-BC77-D2F19A2DED46}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{248DE185-2CE8-4BA6-8D69-F37F45D83A7F}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{248DE185-2CE8-4BA6-8D69-F37F45D83A7F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1878" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1995" uniqueCount="26">
   <si>
     <t>Tissue</t>
   </si>
@@ -112,12 +112,18 @@
   <si>
     <t>Rep2</t>
   </si>
+  <si>
+    <t>MyoG</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="###0.00;\-###0.00"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -130,6 +136,10 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8.25"/>
+      <name val="Microsoft Sans Serif"/>
     </font>
   </fonts>
   <fills count="2">
@@ -152,8 +162,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -488,7 +501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9608A0BB-4834-4C56-8996-87339C4A28ED}">
-  <dimension ref="A1:F625"/>
+  <dimension ref="A1:F664"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="10.7265625" bestFit="1" customWidth="1"/>
@@ -13003,6 +13016,786 @@
         <v>25.75</v>
       </c>
     </row>
+    <row r="626" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A626" t="s">
+        <v>16</v>
+      </c>
+      <c r="B626" t="s">
+        <v>5</v>
+      </c>
+      <c r="C626">
+        <v>1</v>
+      </c>
+      <c r="D626" t="s">
+        <v>25</v>
+      </c>
+      <c r="E626" s="1">
+        <v>28.053165621050098</v>
+      </c>
+      <c r="F626" s="1">
+        <v>28.0857390978917</v>
+      </c>
+    </row>
+    <row r="627" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A627" t="s">
+        <v>16</v>
+      </c>
+      <c r="B627" t="s">
+        <v>5</v>
+      </c>
+      <c r="C627">
+        <v>2</v>
+      </c>
+      <c r="D627" t="s">
+        <v>25</v>
+      </c>
+      <c r="E627" s="1">
+        <v>30.0503992850206</v>
+      </c>
+      <c r="F627" s="1">
+        <v>29.914640295490202</v>
+      </c>
+    </row>
+    <row r="628" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A628" t="s">
+        <v>16</v>
+      </c>
+      <c r="B628" t="s">
+        <v>5</v>
+      </c>
+      <c r="C628">
+        <v>3</v>
+      </c>
+      <c r="D628" t="s">
+        <v>25</v>
+      </c>
+      <c r="E628" s="1">
+        <v>28.808130776376899</v>
+      </c>
+      <c r="F628" s="1">
+        <v>28.576923817220301</v>
+      </c>
+    </row>
+    <row r="629" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A629" t="s">
+        <v>16</v>
+      </c>
+      <c r="B629" t="s">
+        <v>5</v>
+      </c>
+      <c r="C629">
+        <v>4</v>
+      </c>
+      <c r="D629" t="s">
+        <v>25</v>
+      </c>
+      <c r="E629" s="1">
+        <v>28.284978647312801</v>
+      </c>
+      <c r="F629" s="1">
+        <v>27.3132014966417</v>
+      </c>
+    </row>
+    <row r="630" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A630" t="s">
+        <v>16</v>
+      </c>
+      <c r="B630" t="s">
+        <v>5</v>
+      </c>
+      <c r="C630">
+        <v>5</v>
+      </c>
+      <c r="D630" t="s">
+        <v>25</v>
+      </c>
+      <c r="E630" s="1">
+        <v>30.390326192228802</v>
+      </c>
+      <c r="F630" s="1">
+        <v>30.485760002632802</v>
+      </c>
+    </row>
+    <row r="631" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A631" t="s">
+        <v>16</v>
+      </c>
+      <c r="B631" t="s">
+        <v>5</v>
+      </c>
+      <c r="C631">
+        <v>6</v>
+      </c>
+      <c r="D631" t="s">
+        <v>25</v>
+      </c>
+      <c r="E631" s="1">
+        <v>29.053738371678801</v>
+      </c>
+      <c r="F631" s="1">
+        <v>29.515994767132401</v>
+      </c>
+    </row>
+    <row r="632" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A632" t="s">
+        <v>16</v>
+      </c>
+      <c r="B632" t="s">
+        <v>5</v>
+      </c>
+      <c r="C632">
+        <v>7</v>
+      </c>
+      <c r="D632" t="s">
+        <v>25</v>
+      </c>
+      <c r="E632" s="1">
+        <v>29.1718625422718</v>
+      </c>
+      <c r="F632" s="1">
+        <v>29.363604750268301</v>
+      </c>
+    </row>
+    <row r="633" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A633" t="s">
+        <v>16</v>
+      </c>
+      <c r="B633" t="s">
+        <v>5</v>
+      </c>
+      <c r="C633">
+        <v>8</v>
+      </c>
+      <c r="D633" t="s">
+        <v>25</v>
+      </c>
+      <c r="E633" s="1">
+        <v>28.992182255112901</v>
+      </c>
+      <c r="F633" s="1">
+        <v>29.415704724209</v>
+      </c>
+    </row>
+    <row r="634" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A634" t="s">
+        <v>16</v>
+      </c>
+      <c r="B634" t="s">
+        <v>7</v>
+      </c>
+      <c r="C634">
+        <v>1</v>
+      </c>
+      <c r="D634" t="s">
+        <v>25</v>
+      </c>
+      <c r="E634" s="1">
+        <v>29.762943796644201</v>
+      </c>
+      <c r="F634" s="1">
+        <v>30.124111744582098</v>
+      </c>
+    </row>
+    <row r="635" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A635" t="s">
+        <v>16</v>
+      </c>
+      <c r="B635" t="s">
+        <v>7</v>
+      </c>
+      <c r="C635">
+        <v>2</v>
+      </c>
+      <c r="D635" t="s">
+        <v>25</v>
+      </c>
+      <c r="E635" s="1">
+        <v>29.003592063641801</v>
+      </c>
+      <c r="F635" s="1">
+        <v>28.430701827647901</v>
+      </c>
+    </row>
+    <row r="636" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A636" t="s">
+        <v>16</v>
+      </c>
+      <c r="B636" t="s">
+        <v>7</v>
+      </c>
+      <c r="C636">
+        <v>3</v>
+      </c>
+      <c r="D636" t="s">
+        <v>25</v>
+      </c>
+      <c r="E636" s="1">
+        <v>29.5501513232619</v>
+      </c>
+      <c r="F636" s="1">
+        <v>30.608154623024401</v>
+      </c>
+    </row>
+    <row r="637" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A637" t="s">
+        <v>16</v>
+      </c>
+      <c r="B637" t="s">
+        <v>7</v>
+      </c>
+      <c r="C637">
+        <v>4</v>
+      </c>
+      <c r="D637" t="s">
+        <v>25</v>
+      </c>
+      <c r="E637" s="1">
+        <v>33.136986705476403</v>
+      </c>
+      <c r="F637" s="1">
+        <v>32.630932094647903</v>
+      </c>
+    </row>
+    <row r="638" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A638" t="s">
+        <v>16</v>
+      </c>
+      <c r="B638" t="s">
+        <v>7</v>
+      </c>
+      <c r="C638">
+        <v>5</v>
+      </c>
+      <c r="D638" t="s">
+        <v>25</v>
+      </c>
+      <c r="E638" s="1">
+        <v>28.425990012226102</v>
+      </c>
+      <c r="F638" s="1">
+        <v>28.392550644951999</v>
+      </c>
+    </row>
+    <row r="639" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A639" t="s">
+        <v>16</v>
+      </c>
+      <c r="B639" t="s">
+        <v>7</v>
+      </c>
+      <c r="C639">
+        <v>6</v>
+      </c>
+      <c r="D639" t="s">
+        <v>25</v>
+      </c>
+      <c r="E639" s="1">
+        <v>29.4907493719132</v>
+      </c>
+      <c r="F639" s="1">
+        <v>29.533848063526602</v>
+      </c>
+    </row>
+    <row r="640" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A640" t="s">
+        <v>16</v>
+      </c>
+      <c r="B640" t="s">
+        <v>7</v>
+      </c>
+      <c r="C640">
+        <v>7</v>
+      </c>
+      <c r="D640" t="s">
+        <v>25</v>
+      </c>
+      <c r="E640" s="1">
+        <v>29.704909939280899</v>
+      </c>
+      <c r="F640" s="1">
+        <v>30.357917384956199</v>
+      </c>
+    </row>
+    <row r="641" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A641" t="s">
+        <v>16</v>
+      </c>
+      <c r="B641" t="s">
+        <v>8</v>
+      </c>
+      <c r="C641">
+        <v>1</v>
+      </c>
+      <c r="D641" t="s">
+        <v>25</v>
+      </c>
+      <c r="E641" s="1">
+        <v>27.168407914522099</v>
+      </c>
+      <c r="F641" s="1">
+        <v>27.6536793442815</v>
+      </c>
+    </row>
+    <row r="642" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A642" t="s">
+        <v>16</v>
+      </c>
+      <c r="B642" t="s">
+        <v>8</v>
+      </c>
+      <c r="C642">
+        <v>2</v>
+      </c>
+      <c r="D642" t="s">
+        <v>25</v>
+      </c>
+      <c r="E642" s="1">
+        <v>27.609675486490001</v>
+      </c>
+      <c r="F642" s="1">
+        <v>26.964926728312399</v>
+      </c>
+    </row>
+    <row r="643" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A643" t="s">
+        <v>16</v>
+      </c>
+      <c r="B643" t="s">
+        <v>8</v>
+      </c>
+      <c r="C643">
+        <v>3</v>
+      </c>
+      <c r="D643" t="s">
+        <v>25</v>
+      </c>
+      <c r="E643" s="1">
+        <v>28.144459995911301</v>
+      </c>
+      <c r="F643" s="1">
+        <v>28.764965480241798</v>
+      </c>
+    </row>
+    <row r="644" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A644" t="s">
+        <v>16</v>
+      </c>
+      <c r="B644" t="s">
+        <v>8</v>
+      </c>
+      <c r="C644">
+        <v>4</v>
+      </c>
+      <c r="D644" t="s">
+        <v>25</v>
+      </c>
+      <c r="E644" s="1">
+        <v>27.182718432696198</v>
+      </c>
+      <c r="F644" s="1">
+        <v>27.336956639467399</v>
+      </c>
+    </row>
+    <row r="645" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A645" t="s">
+        <v>16</v>
+      </c>
+      <c r="B645" t="s">
+        <v>8</v>
+      </c>
+      <c r="C645">
+        <v>5</v>
+      </c>
+      <c r="D645" t="s">
+        <v>25</v>
+      </c>
+      <c r="E645" s="1">
+        <v>27.918984886755499</v>
+      </c>
+      <c r="F645" s="1">
+        <v>28.173490594127699</v>
+      </c>
+    </row>
+    <row r="646" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A646" t="s">
+        <v>16</v>
+      </c>
+      <c r="B646" t="s">
+        <v>8</v>
+      </c>
+      <c r="C646">
+        <v>6</v>
+      </c>
+      <c r="D646" t="s">
+        <v>25</v>
+      </c>
+      <c r="E646" s="1">
+        <v>28.891312906224702</v>
+      </c>
+      <c r="F646" s="1">
+        <v>29.148843631370099</v>
+      </c>
+    </row>
+    <row r="647" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A647" t="s">
+        <v>16</v>
+      </c>
+      <c r="B647" t="s">
+        <v>8</v>
+      </c>
+      <c r="C647">
+        <v>7</v>
+      </c>
+      <c r="D647" t="s">
+        <v>25</v>
+      </c>
+      <c r="E647" s="1">
+        <v>28.011845115892399</v>
+      </c>
+      <c r="F647" s="1">
+        <v>28.185080985237398</v>
+      </c>
+    </row>
+    <row r="648" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A648" t="s">
+        <v>16</v>
+      </c>
+      <c r="B648" t="s">
+        <v>8</v>
+      </c>
+      <c r="C648">
+        <v>8</v>
+      </c>
+      <c r="D648" t="s">
+        <v>25</v>
+      </c>
+      <c r="E648" s="1">
+        <v>27.6476583637108</v>
+      </c>
+      <c r="F648" s="1">
+        <v>28.067250069473499</v>
+      </c>
+    </row>
+    <row r="649" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A649" t="s">
+        <v>16</v>
+      </c>
+      <c r="B649" t="s">
+        <v>9</v>
+      </c>
+      <c r="C649">
+        <v>1</v>
+      </c>
+      <c r="D649" t="s">
+        <v>25</v>
+      </c>
+      <c r="E649" s="1">
+        <v>33.102216295024199</v>
+      </c>
+      <c r="F649" s="1">
+        <v>33.104510385428803</v>
+      </c>
+    </row>
+    <row r="650" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A650" t="s">
+        <v>16</v>
+      </c>
+      <c r="B650" t="s">
+        <v>9</v>
+      </c>
+      <c r="C650">
+        <v>2</v>
+      </c>
+      <c r="D650" t="s">
+        <v>25</v>
+      </c>
+      <c r="E650" s="1">
+        <v>27.813685509001399</v>
+      </c>
+      <c r="F650" s="1">
+        <v>27.786019371039401</v>
+      </c>
+    </row>
+    <row r="651" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A651" t="s">
+        <v>16</v>
+      </c>
+      <c r="B651" t="s">
+        <v>9</v>
+      </c>
+      <c r="C651">
+        <v>3</v>
+      </c>
+      <c r="D651" t="s">
+        <v>25</v>
+      </c>
+      <c r="E651" s="1">
+        <v>27.0002496869593</v>
+      </c>
+      <c r="F651" s="1">
+        <v>27.048263111997301</v>
+      </c>
+    </row>
+    <row r="652" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A652" t="s">
+        <v>16</v>
+      </c>
+      <c r="B652" t="s">
+        <v>9</v>
+      </c>
+      <c r="C652">
+        <v>4</v>
+      </c>
+      <c r="D652" t="s">
+        <v>25</v>
+      </c>
+      <c r="E652" s="1">
+        <v>26.914111002612199</v>
+      </c>
+      <c r="F652" s="1">
+        <v>26.680127577512302</v>
+      </c>
+    </row>
+    <row r="653" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A653" t="s">
+        <v>16</v>
+      </c>
+      <c r="B653" t="s">
+        <v>9</v>
+      </c>
+      <c r="C653">
+        <v>5</v>
+      </c>
+      <c r="D653" t="s">
+        <v>25</v>
+      </c>
+      <c r="E653" s="1">
+        <v>26.219470282299099</v>
+      </c>
+      <c r="F653" s="1">
+        <v>26.061908314495899</v>
+      </c>
+    </row>
+    <row r="654" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A654" t="s">
+        <v>16</v>
+      </c>
+      <c r="B654" t="s">
+        <v>9</v>
+      </c>
+      <c r="C654">
+        <v>6</v>
+      </c>
+      <c r="D654" t="s">
+        <v>25</v>
+      </c>
+      <c r="E654" s="1">
+        <v>26.713019766875899</v>
+      </c>
+      <c r="F654" s="1">
+        <v>26.591890124942001</v>
+      </c>
+    </row>
+    <row r="655" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A655" t="s">
+        <v>16</v>
+      </c>
+      <c r="B655" t="s">
+        <v>9</v>
+      </c>
+      <c r="C655">
+        <v>7</v>
+      </c>
+      <c r="D655" t="s">
+        <v>25</v>
+      </c>
+      <c r="E655" s="1">
+        <v>28.341086290718099</v>
+      </c>
+      <c r="F655" s="1">
+        <v>28.133909413643501</v>
+      </c>
+    </row>
+    <row r="656" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A656" t="s">
+        <v>16</v>
+      </c>
+      <c r="B656" t="s">
+        <v>9</v>
+      </c>
+      <c r="C656">
+        <v>8</v>
+      </c>
+      <c r="D656" t="s">
+        <v>25</v>
+      </c>
+      <c r="E656" s="1">
+        <v>25.840218410083899</v>
+      </c>
+      <c r="F656" s="1">
+        <v>26.463865557737702</v>
+      </c>
+    </row>
+    <row r="657" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A657" t="s">
+        <v>16</v>
+      </c>
+      <c r="B657" t="s">
+        <v>10</v>
+      </c>
+      <c r="C657">
+        <v>1</v>
+      </c>
+      <c r="D657" t="s">
+        <v>25</v>
+      </c>
+      <c r="E657" s="1">
+        <v>27.398366465647001</v>
+      </c>
+      <c r="F657" s="1">
+        <v>27.102292986943301</v>
+      </c>
+    </row>
+    <row r="658" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A658" t="s">
+        <v>16</v>
+      </c>
+      <c r="B658" t="s">
+        <v>10</v>
+      </c>
+      <c r="C658">
+        <v>2</v>
+      </c>
+      <c r="D658" t="s">
+        <v>25</v>
+      </c>
+      <c r="E658" s="1">
+        <v>26.850115891102799</v>
+      </c>
+      <c r="F658" s="1">
+        <v>26.795560367619</v>
+      </c>
+    </row>
+    <row r="659" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A659" t="s">
+        <v>16</v>
+      </c>
+      <c r="B659" t="s">
+        <v>10</v>
+      </c>
+      <c r="C659">
+        <v>3</v>
+      </c>
+      <c r="D659" t="s">
+        <v>25</v>
+      </c>
+      <c r="E659" s="1">
+        <v>26.556454031254798</v>
+      </c>
+      <c r="F659" s="1">
+        <v>26.438626892519199</v>
+      </c>
+    </row>
+    <row r="660" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A660" t="s">
+        <v>16</v>
+      </c>
+      <c r="B660" t="s">
+        <v>10</v>
+      </c>
+      <c r="C660">
+        <v>4</v>
+      </c>
+      <c r="D660" t="s">
+        <v>25</v>
+      </c>
+      <c r="E660" s="1">
+        <v>26.295859854968199</v>
+      </c>
+      <c r="F660" s="1">
+        <v>26.315415922219699</v>
+      </c>
+    </row>
+    <row r="661" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A661" t="s">
+        <v>16</v>
+      </c>
+      <c r="B661" t="s">
+        <v>10</v>
+      </c>
+      <c r="C661">
+        <v>5</v>
+      </c>
+      <c r="D661" t="s">
+        <v>25</v>
+      </c>
+      <c r="E661" s="1">
+        <v>26.448558098527801</v>
+      </c>
+      <c r="F661" s="1">
+        <v>26.341777016003</v>
+      </c>
+    </row>
+    <row r="662" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A662" t="s">
+        <v>16</v>
+      </c>
+      <c r="B662" t="s">
+        <v>10</v>
+      </c>
+      <c r="C662">
+        <v>6</v>
+      </c>
+      <c r="D662" t="s">
+        <v>25</v>
+      </c>
+      <c r="E662" s="1">
+        <v>26.8968557141418</v>
+      </c>
+      <c r="F662" s="1">
+        <v>26.675821102362899</v>
+      </c>
+    </row>
+    <row r="663" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A663" t="s">
+        <v>16</v>
+      </c>
+      <c r="B663" t="s">
+        <v>10</v>
+      </c>
+      <c r="C663">
+        <v>7</v>
+      </c>
+      <c r="D663" t="s">
+        <v>25</v>
+      </c>
+      <c r="E663" s="1">
+        <v>26.190511241868499</v>
+      </c>
+      <c r="F663" s="1">
+        <v>26.071947071713101</v>
+      </c>
+    </row>
+    <row r="664" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A664" t="s">
+        <v>16</v>
+      </c>
+      <c r="B664" t="s">
+        <v>10</v>
+      </c>
+      <c r="C664">
+        <v>8</v>
+      </c>
+      <c r="D664" t="s">
+        <v>25</v>
+      </c>
+      <c r="E664" s="1">
+        <v>26.186975051831801</v>
+      </c>
+      <c r="F664" s="1">
+        <v>26.1776042433413</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>